<commit_message>
운동프로그램 갱신 2026-08-28  9:41:51.75
</commit_message>
<xml_diff>
--- a/운동프로그램_8일주기_v19.xlsx
+++ b/운동프로그램_8일주기_v19.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_AD191220E1AB09E8313BB3B3DC196F42CA207056" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_AD191220E1AB09E8313BB3B3DC196F42CA207056" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDA99C23-B7BB-451B-86B7-1EB9C7BFDDF3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="883" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1726,9 +1726,6 @@
     <t>가장 작은 근육군 — 절대값이 작아 2.25kg은 과함</t>
   </si>
   <si>
-    <t>날짜</t>
-  </si>
-  <si>
     <t>스쿼트 목표</t>
   </si>
   <si>
@@ -2351,6 +2348,10 @@
   </si>
   <si>
     <t>· 쌓는 시기와 지키는 시기는 다르게 설계해야 한다.</t>
+  </si>
+  <si>
+    <t>날짜 (1일차)</t>
+    <phoneticPr fontId="34" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -2731,7 +2732,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="36" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2968,6 +2969,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -4847,7 +4851,7 @@
         <v>1</v>
       </c>
       <c r="F39" s="52">
-        <f t="shared" ref="F39:F70" ca="1" si="3">IF(ISNUMBER(E39),$D39*E39,0)</f>
+        <f t="shared" ref="F39:F61" ca="1" si="3">IF(ISNUMBER(E39),$D39*E39,0)</f>
         <v>0</v>
       </c>
       <c r="G39" s="56" t="s">
@@ -6376,31 +6380,31 @@
         <v>98</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>766</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>558</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="D9" s="5" t="s">
         <v>559</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="E9" s="5" t="s">
         <v>560</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="F9" s="5" t="s">
+        <v>559</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>561</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>560</v>
-      </c>
-      <c r="G9" s="5" t="s">
+      <c r="H9" s="5" t="s">
+        <v>559</v>
+      </c>
+      <c r="I9" s="5" t="s">
         <v>562</v>
       </c>
-      <c r="H9" s="5" t="s">
-        <v>560</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>563</v>
-      </c>
       <c r="J9" s="5" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="K9" s="5" t="s">
         <v>16</v>
@@ -6491,7 +6495,9 @@
       <c r="A13" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="B13" s="4"/>
+      <c r="B13" s="96">
+        <v>46262</v>
+      </c>
       <c r="C13" s="16">
         <f t="shared" si="0"/>
         <v>52.5</v>
@@ -6732,17 +6738,17 @@
     </row>
     <row r="23" spans="1:11" ht="108" customHeight="1">
       <c r="A23" s="11" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="84" customHeight="1">
       <c r="A24" s="11" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
     </row>
     <row r="25" spans="1:11" ht="84" customHeight="1">
       <c r="A25" s="11" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
     </row>
     <row r="26" spans="1:11" ht="120" customHeight="1">
@@ -6750,27 +6756,27 @@
     </row>
     <row r="27" spans="1:11" ht="96" customHeight="1">
       <c r="A27" s="11" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
     </row>
     <row r="28" spans="1:11" ht="108" customHeight="1">
       <c r="A28" s="11" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="108" customHeight="1">
       <c r="A29" s="11" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="156" customHeight="1">
       <c r="A30" s="11" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="96" customHeight="1">
       <c r="A31" s="11" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
   </sheetData>
@@ -6791,23 +6797,23 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18" customHeight="1">
       <c r="A1" s="71" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15" customHeight="1">
       <c r="A4" s="5" t="s">
+        <v>573</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>574</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5" t="s">
         <v>575</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>576</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15" customHeight="1">
@@ -6815,21 +6821,21 @@
         <v>507</v>
       </c>
       <c r="B5" s="7" t="s">
+        <v>576</v>
+      </c>
+      <c r="C5" s="58" t="s">
         <v>577</v>
-      </c>
-      <c r="C5" s="58" t="s">
-        <v>578</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="15" customHeight="1">
       <c r="A6" s="7" t="s">
+        <v>578</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>576</v>
+      </c>
+      <c r="C6" s="58" t="s">
         <v>579</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>577</v>
-      </c>
-      <c r="C6" s="58" t="s">
-        <v>580</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="15" customHeight="1">
@@ -6837,80 +6843,80 @@
         <v>235</v>
       </c>
       <c r="B7" s="7" t="s">
+        <v>580</v>
+      </c>
+      <c r="C7" s="58" t="s">
         <v>581</v>
-      </c>
-      <c r="C7" s="58" t="s">
-        <v>582</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="15" customHeight="1">
       <c r="A8" s="72" t="s">
+        <v>582</v>
+      </c>
+      <c r="B8" s="72" t="s">
         <v>583</v>
       </c>
-      <c r="B8" s="72" t="s">
+      <c r="C8" s="73" t="s">
         <v>584</v>
-      </c>
-      <c r="C8" s="73" t="s">
-        <v>585</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15" customHeight="1">
       <c r="A9" s="72" t="s">
+        <v>585</v>
+      </c>
+      <c r="B9" s="72" t="s">
+        <v>583</v>
+      </c>
+      <c r="C9" s="73" t="s">
         <v>586</v>
-      </c>
-      <c r="B9" s="72" t="s">
-        <v>584</v>
-      </c>
-      <c r="C9" s="73" t="s">
-        <v>587</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15" customHeight="1">
       <c r="A10" s="7" t="s">
+        <v>587</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>588</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="C10" s="74" t="s">
         <v>589</v>
-      </c>
-      <c r="C10" s="74" t="s">
-        <v>590</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="15" customHeight="1">
       <c r="A11" s="7" t="s">
+        <v>590</v>
+      </c>
+      <c r="B11" s="8" t="s">
         <v>591</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="C11" s="58" t="s">
         <v>592</v>
-      </c>
-      <c r="C11" s="58" t="s">
-        <v>593</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="15" customHeight="1">
       <c r="A12" s="7" t="s">
+        <v>593</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>594</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="C12" s="58" t="s">
         <v>595</v>
-      </c>
-      <c r="C12" s="58" t="s">
-        <v>596</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="24" customHeight="1">
       <c r="A15" s="11" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="24" customHeight="1">
       <c r="A16" s="11" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="36" customHeight="1">
       <c r="A17" s="11" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="15" customHeight="1">
@@ -6918,47 +6924,47 @@
     </row>
     <row r="19" spans="1:1" ht="36" customHeight="1">
       <c r="A19" s="11" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="36" customHeight="1">
       <c r="A20" s="11" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="48" customHeight="1">
       <c r="A22" s="13" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="16.5" customHeight="1">
       <c r="A24" s="14" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="16.5" customHeight="1">
       <c r="A25" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="16.5" customHeight="1">
       <c r="A26" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="16.5" customHeight="1">
       <c r="A27" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
     </row>
     <row r="28" spans="1:1" ht="16.5" customHeight="1">
       <c r="A28" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="16.5" customHeight="1">
       <c r="A30" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
     </row>
   </sheetData>
@@ -6982,48 +6988,48 @@
   <sheetData>
     <row r="1" spans="1:6" ht="17.25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1">
       <c r="A2" s="75" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
     </row>
     <row r="3" spans="1:6" ht="16.5" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1">
       <c r="A5" s="5" t="s">
+        <v>611</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>612</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="5" t="s">
         <v>613</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>614</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>615</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>5</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1">
       <c r="A6" s="76" t="s">
+        <v>616</v>
+      </c>
+      <c r="B6" s="77" t="s">
         <v>617</v>
       </c>
-      <c r="B6" s="77" t="s">
-        <v>618</v>
-      </c>
       <c r="C6" s="77" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D6" s="76" t="s">
         <v>134</v>
@@ -7032,39 +7038,39 @@
         <v>0</v>
       </c>
       <c r="F6" s="78" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="15" customHeight="1">
       <c r="A7" s="7" t="s">
+        <v>619</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>617</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>617</v>
+      </c>
+      <c r="D7" s="72" t="s">
         <v>620</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>618</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>618</v>
-      </c>
-      <c r="D7" s="72" t="s">
-        <v>621</v>
       </c>
       <c r="E7" s="7">
         <f>복귀_화_상체밀기!$E$11</f>
         <v>22</v>
       </c>
       <c r="F7" s="74" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="15" customHeight="1">
       <c r="A8" s="76" t="s">
+        <v>622</v>
+      </c>
+      <c r="B8" s="77" t="s">
         <v>623</v>
       </c>
-      <c r="B8" s="77" t="s">
-        <v>624</v>
-      </c>
       <c r="C8" s="77" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="D8" s="76" t="s">
         <v>134</v>
@@ -7073,18 +7079,18 @@
         <v>0</v>
       </c>
       <c r="F8" s="78" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="15" customHeight="1">
       <c r="A9" s="76" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="B9" s="77" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="C9" s="77" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D9" s="76" t="s">
         <v>134</v>
@@ -7093,18 +7099,18 @@
         <v>0</v>
       </c>
       <c r="F9" s="78" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="15" customHeight="1">
       <c r="A10" s="76" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="B10" s="77" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="C10" s="77" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="D10" s="76" t="s">
         <v>134</v>
@@ -7113,39 +7119,39 @@
         <v>0</v>
       </c>
       <c r="F10" s="78" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1">
       <c r="A11" s="7" t="s">
+        <v>629</v>
+      </c>
+      <c r="B11" s="7" t="s">
         <v>630</v>
       </c>
-      <c r="B11" s="7" t="s">
-        <v>631</v>
-      </c>
       <c r="C11" s="7" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="D11" s="72" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="E11" s="7">
         <f>복귀_토_하체!$E$12</f>
         <v>22</v>
       </c>
       <c r="F11" s="58" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="15" customHeight="1">
       <c r="A12" s="7" t="s">
+        <v>632</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>633</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>634</v>
-      </c>
       <c r="C12" s="7" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="D12" s="72" t="s">
         <v>507</v>
@@ -7155,7 +7161,7 @@
         <v>22</v>
       </c>
       <c r="F12" s="58" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15" customHeight="1">
@@ -7173,27 +7179,27 @@
     </row>
     <row r="15" spans="1:6" ht="48" customHeight="1">
       <c r="A15" s="13" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="141" customHeight="1">
       <c r="A16" s="11" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="126" customHeight="1">
       <c r="A17" s="11" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="77.25" customHeight="1">
       <c r="A18" s="11" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="115.5" customHeight="1">
       <c r="A19" s="11" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="15" customHeight="1">
@@ -7201,32 +7207,32 @@
     </row>
     <row r="21" spans="1:1" ht="48" customHeight="1">
       <c r="A21" s="13" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="141" customHeight="1">
       <c r="A22" s="11" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="77.25" customHeight="1">
       <c r="A23" s="11" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="24" spans="1:1" ht="90" customHeight="1">
       <c r="A24" s="11" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="128.25" customHeight="1">
       <c r="A25" s="11" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="26" spans="1:1" ht="128.25" customHeight="1">
       <c r="A26" s="11" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
     </row>
     <row r="27" spans="1:1" ht="15" customHeight="1">
@@ -7234,37 +7240,37 @@
     </row>
     <row r="28" spans="1:1" ht="48" customHeight="1">
       <c r="A28" s="13" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
     </row>
     <row r="29" spans="1:1" ht="75" customHeight="1">
       <c r="A29" s="11" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
     </row>
     <row r="30" spans="1:1" ht="102.75" customHeight="1">
       <c r="A30" s="11" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
     </row>
     <row r="31" spans="1:1" ht="90" customHeight="1">
       <c r="A31" s="11" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
     </row>
     <row r="32" spans="1:1" ht="128.25" customHeight="1">
       <c r="A32" s="11" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
     </row>
     <row r="33" spans="1:1" ht="144" customHeight="1">
       <c r="A33" s="11" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
     </row>
     <row r="34" spans="1:1" ht="15" customHeight="1">
       <c r="A34" s="79" t="s">
-        <v>653</v>
+        <v>652</v>
       </c>
     </row>
   </sheetData>
@@ -7291,12 +7297,12 @@
   <sheetData>
     <row r="1" spans="1:8" ht="21" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>654</v>
+        <v>653</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
@@ -7346,10 +7352,10 @@
         <v>20</v>
       </c>
       <c r="G5" s="73" t="s">
+        <v>655</v>
+      </c>
+      <c r="H5" s="73" t="s">
         <v>656</v>
-      </c>
-      <c r="H5" s="73" t="s">
-        <v>657</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -7363,7 +7369,7 @@
         <v>249</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="E6" s="7">
         <v>3</v>
@@ -7372,10 +7378,10 @@
         <v>25</v>
       </c>
       <c r="G6" s="58" t="s">
+        <v>658</v>
+      </c>
+      <c r="H6" s="58" t="s">
         <v>659</v>
-      </c>
-      <c r="H6" s="58" t="s">
-        <v>660</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1">
@@ -7389,7 +7395,7 @@
         <v>258</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>661</v>
+        <v>660</v>
       </c>
       <c r="E7" s="7">
         <v>3</v>
@@ -7398,10 +7404,10 @@
         <v>208</v>
       </c>
       <c r="G7" s="58" t="s">
+        <v>661</v>
+      </c>
+      <c r="H7" s="58" t="s">
         <v>662</v>
-      </c>
-      <c r="H7" s="58" t="s">
-        <v>663</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1">
@@ -7424,10 +7430,10 @@
         <v>25</v>
       </c>
       <c r="G8" s="58" t="s">
+        <v>663</v>
+      </c>
+      <c r="H8" s="58" t="s">
         <v>664</v>
-      </c>
-      <c r="H8" s="58" t="s">
-        <v>665</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1">
@@ -7450,10 +7456,10 @@
         <v>42</v>
       </c>
       <c r="G9" s="58" t="s">
+        <v>665</v>
+      </c>
+      <c r="H9" s="58" t="s">
         <v>666</v>
-      </c>
-      <c r="H9" s="58" t="s">
-        <v>667</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1">
@@ -7476,10 +7482,10 @@
         <v>42</v>
       </c>
       <c r="G10" s="58" t="s">
+        <v>667</v>
+      </c>
+      <c r="H10" s="58" t="s">
         <v>668</v>
-      </c>
-      <c r="H10" s="58" t="s">
-        <v>669</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -7493,22 +7499,22 @@
     </row>
     <row r="13" spans="1:8" ht="32.25" customHeight="1">
       <c r="A13" s="12" t="s">
-        <v>670</v>
+        <v>669</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="278.25" customHeight="1">
       <c r="A14" s="11" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="237.75" customHeight="1">
       <c r="A15" s="11" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="237.75" customHeight="1">
       <c r="A16" s="11" t="s">
-        <v>673</v>
+        <v>672</v>
       </c>
     </row>
   </sheetData>
@@ -7535,12 +7541,12 @@
   <sheetData>
     <row r="1" spans="1:8" ht="21" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>674</v>
+        <v>673</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>675</v>
+        <v>674</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
@@ -7590,10 +7596,10 @@
         <v>5</v>
       </c>
       <c r="G5" s="73" t="s">
+        <v>675</v>
+      </c>
+      <c r="H5" s="73" t="s">
         <v>676</v>
-      </c>
-      <c r="H5" s="73" t="s">
-        <v>677</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="29.25" customHeight="1">
@@ -7616,10 +7622,10 @@
         <v>25</v>
       </c>
       <c r="G6" s="73" t="s">
+        <v>677</v>
+      </c>
+      <c r="H6" s="73" t="s">
         <v>678</v>
-      </c>
-      <c r="H6" s="73" t="s">
-        <v>679</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1">
@@ -7642,10 +7648,10 @@
         <v>37</v>
       </c>
       <c r="G7" s="58" t="s">
+        <v>679</v>
+      </c>
+      <c r="H7" s="58" t="s">
         <v>680</v>
-      </c>
-      <c r="H7" s="58" t="s">
-        <v>681</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1">
@@ -7668,10 +7674,10 @@
         <v>37</v>
       </c>
       <c r="G8" s="58" t="s">
+        <v>681</v>
+      </c>
+      <c r="H8" s="58" t="s">
         <v>682</v>
-      </c>
-      <c r="H8" s="58" t="s">
-        <v>683</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1">
@@ -7694,10 +7700,10 @@
         <v>10</v>
       </c>
       <c r="G9" s="58" t="s">
+        <v>683</v>
+      </c>
+      <c r="H9" s="58" t="s">
         <v>684</v>
-      </c>
-      <c r="H9" s="58" t="s">
-        <v>685</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1">
@@ -7720,10 +7726,10 @@
         <v>42</v>
       </c>
       <c r="G10" s="58" t="s">
+        <v>685</v>
+      </c>
+      <c r="H10" s="58" t="s">
         <v>686</v>
-      </c>
-      <c r="H10" s="58" t="s">
-        <v>687</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -7731,7 +7737,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="58" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="C11" s="7" t="s">
         <v>313</v>
@@ -7747,10 +7753,10 @@
         <v>5</v>
       </c>
       <c r="G11" s="58" t="s">
+        <v>688</v>
+      </c>
+      <c r="H11" s="58" t="s">
         <v>689</v>
-      </c>
-      <c r="H11" s="58" t="s">
-        <v>690</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -7764,22 +7770,22 @@
     </row>
     <row r="14" spans="1:8" ht="76.5" customHeight="1">
       <c r="A14" s="12" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="265.5" customHeight="1">
       <c r="A15" s="11" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="293.25" customHeight="1">
       <c r="A16" s="11" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="276" customHeight="1">
       <c r="A17" s="11" t="s">
-        <v>694</v>
+        <v>693</v>
       </c>
     </row>
   </sheetData>
@@ -7806,12 +7812,12 @@
   <sheetData>
     <row r="1" spans="1:8" ht="21" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="15" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="15" customHeight="1">
@@ -7861,10 +7867,10 @@
         <v>5</v>
       </c>
       <c r="G5" s="73" t="s">
+        <v>696</v>
+      </c>
+      <c r="H5" s="73" t="s">
         <v>697</v>
-      </c>
-      <c r="H5" s="73" t="s">
-        <v>698</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -7887,10 +7893,10 @@
         <v>208</v>
       </c>
       <c r="G6" s="58" t="s">
+        <v>698</v>
+      </c>
+      <c r="H6" s="58" t="s">
         <v>699</v>
-      </c>
-      <c r="H6" s="58" t="s">
-        <v>700</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15" customHeight="1">
@@ -7913,10 +7919,10 @@
         <v>25</v>
       </c>
       <c r="G7" s="58" t="s">
+        <v>700</v>
+      </c>
+      <c r="H7" s="58" t="s">
         <v>701</v>
-      </c>
-      <c r="H7" s="58" t="s">
-        <v>702</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15" customHeight="1">
@@ -7939,10 +7945,10 @@
         <v>200</v>
       </c>
       <c r="G8" s="58" t="s">
+        <v>702</v>
+      </c>
+      <c r="H8" s="58" t="s">
         <v>703</v>
-      </c>
-      <c r="H8" s="58" t="s">
-        <v>704</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15" customHeight="1">
@@ -7965,10 +7971,10 @@
         <v>25</v>
       </c>
       <c r="G9" s="58" t="s">
+        <v>704</v>
+      </c>
+      <c r="H9" s="58" t="s">
         <v>705</v>
-      </c>
-      <c r="H9" s="58" t="s">
-        <v>706</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15" customHeight="1">
@@ -7991,10 +7997,10 @@
         <v>42</v>
       </c>
       <c r="G10" s="58" t="s">
+        <v>706</v>
+      </c>
+      <c r="H10" s="58" t="s">
         <v>707</v>
-      </c>
-      <c r="H10" s="58" t="s">
-        <v>708</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -8017,10 +8023,10 @@
         <v>25</v>
       </c>
       <c r="G11" s="58" t="s">
+        <v>708</v>
+      </c>
+      <c r="H11" s="58" t="s">
         <v>709</v>
-      </c>
-      <c r="H11" s="58" t="s">
-        <v>710</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -8028,7 +8034,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="58" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="C12" s="7" t="s">
         <v>56</v>
@@ -8043,10 +8049,10 @@
         <v>12</v>
       </c>
       <c r="G12" s="58" t="s">
+        <v>711</v>
+      </c>
+      <c r="H12" s="58" t="s">
         <v>712</v>
-      </c>
-      <c r="H12" s="58" t="s">
-        <v>713</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="15" customHeight="1">
@@ -8060,22 +8066,22 @@
     </row>
     <row r="15" spans="1:8" ht="92.25" customHeight="1">
       <c r="A15" s="12" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="233.25" customHeight="1">
       <c r="A16" s="11" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="240" customHeight="1">
       <c r="A17" s="11" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="278.25" customHeight="1">
       <c r="A18" s="11" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="15" customHeight="1">
@@ -8083,12 +8089,12 @@
     </row>
     <row r="20" spans="1:1" ht="95.25" customHeight="1">
       <c r="A20" s="12" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="21" spans="1:1" ht="252.75" customHeight="1">
       <c r="A21" s="11" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="237.75" customHeight="1">
@@ -8096,7 +8102,7 @@
     </row>
     <row r="23" spans="1:1" ht="265.5" customHeight="1">
       <c r="A23" s="11" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
     </row>
   </sheetData>
@@ -8118,96 +8124,96 @@
   <sheetData>
     <row r="1" spans="1:4" ht="17.25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1">
       <c r="A4" s="5" t="s">
+        <v>722</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>723</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5" t="s">
         <v>724</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>725</v>
-      </c>
       <c r="D4" s="5" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15" customHeight="1">
       <c r="A5" s="7" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="B5" s="7" t="s">
+        <v>725</v>
+      </c>
+      <c r="C5" s="7" t="s">
         <v>726</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="D5" s="74" t="s">
         <v>727</v>
-      </c>
-      <c r="D5" s="74" t="s">
-        <v>728</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15" customHeight="1">
       <c r="A6" s="7" t="s">
+        <v>728</v>
+      </c>
+      <c r="B6" s="8" t="s">
         <v>729</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>730</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="D6" s="58" t="s">
         <v>731</v>
-      </c>
-      <c r="D6" s="58" t="s">
-        <v>732</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15" customHeight="1">
       <c r="A7" s="7" t="s">
+        <v>732</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>733</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="7" t="s">
         <v>734</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="D7" s="58" t="s">
         <v>735</v>
-      </c>
-      <c r="D7" s="58" t="s">
-        <v>736</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15" customHeight="1">
       <c r="A8" s="7" t="s">
+        <v>736</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>737</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="C8" s="7" t="s">
         <v>738</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="D8" s="58" t="s">
         <v>739</v>
-      </c>
-      <c r="D8" s="58" t="s">
-        <v>740</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15" customHeight="1">
       <c r="A9" s="7" t="s">
+        <v>740</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>741</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="C9" s="8" t="s">
         <v>742</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="D9" s="58" t="s">
         <v>743</v>
-      </c>
-      <c r="D9" s="58" t="s">
-        <v>744</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15" customHeight="1">
@@ -8215,13 +8221,13 @@
         <v>71</v>
       </c>
       <c r="B10" s="8" t="s">
+        <v>744</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>745</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="D10" s="58" t="s">
         <v>746</v>
-      </c>
-      <c r="D10" s="58" t="s">
-        <v>747</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15" customHeight="1">
@@ -8229,66 +8235,66 @@
         <v>69</v>
       </c>
       <c r="B11" s="8" t="s">
+        <v>747</v>
+      </c>
+      <c r="C11" s="8" t="s">
         <v>748</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="D11" s="58" t="s">
         <v>749</v>
-      </c>
-      <c r="D11" s="58" t="s">
-        <v>750</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15" customHeight="1">
       <c r="A12" s="7" t="s">
+        <v>750</v>
+      </c>
+      <c r="B12" s="8" t="s">
         <v>751</v>
       </c>
-      <c r="B12" s="8" t="s">
+      <c r="C12" s="8" t="s">
         <v>752</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="D12" s="58" t="s">
         <v>753</v>
-      </c>
-      <c r="D12" s="58" t="s">
-        <v>754</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15" customHeight="1">
       <c r="A13" s="84" t="s">
+        <v>754</v>
+      </c>
+      <c r="B13" s="85" t="s">
         <v>755</v>
       </c>
-      <c r="B13" s="85" t="s">
+      <c r="C13" s="85" t="s">
         <v>756</v>
       </c>
-      <c r="C13" s="85" t="s">
+      <c r="D13" s="84" t="s">
         <v>757</v>
-      </c>
-      <c r="D13" s="84" t="s">
-        <v>758</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15" customHeight="1">
       <c r="A15" s="3" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="39" customHeight="1">
       <c r="A16" s="11" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
     </row>
     <row r="17" spans="1:1" ht="51.75" customHeight="1">
       <c r="A17" s="11" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="18" spans="1:1" ht="39" customHeight="1">
       <c r="A18" s="11" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="19" spans="1:1" ht="39" customHeight="1">
       <c r="A19" s="11" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="20" spans="1:1" ht="15" customHeight="1">
@@ -8296,12 +8302,12 @@
     </row>
     <row r="21" spans="1:1" ht="51.75" customHeight="1">
       <c r="A21" s="11" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
     </row>
     <row r="22" spans="1:1" ht="39" customHeight="1">
       <c r="A22" s="11" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
     </row>
     <row r="23" spans="1:1" ht="15" customHeight="1">
@@ -8309,12 +8315,12 @@
     </row>
     <row r="24" spans="1:1" ht="51.75" customHeight="1">
       <c r="A24" s="11" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
     </row>
     <row r="25" spans="1:1" ht="39" customHeight="1">
       <c r="A25" s="11" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
운동프로그램 갱신 2026-08-28  9:51:03.16
</commit_message>
<xml_diff>
--- a/운동프로그램_8일주기_v19.xlsx
+++ b/운동프로그램_8일주기_v19.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b2bc197408547891/Desktop/운동/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_AD191220E1AB09E8313BB3B3DC196F42CA207056" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FDA99C23-B7BB-451B-86B7-1EB9C7BFDDF3}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_AD191220E1AB09E8313BB3B3DC196F42CA207056" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9D6C4A2A-567C-4197-B8FB-CADAF6883FC7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="883" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2958,6 +2958,9 @@
     </xf>
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2969,9 +2972,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -3144,6 +3144,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3888,28 +3892,28 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
-      <c r="A2" s="93" t="s">
+      <c r="A2" s="94" t="s">
         <v>424</v>
       </c>
-      <c r="B2" s="92"/>
-      <c r="C2" s="92"/>
-      <c r="D2" s="92"/>
-      <c r="E2" s="92"/>
-      <c r="F2" s="92"/>
-      <c r="G2" s="92"/>
-      <c r="H2" s="92"/>
+      <c r="B2" s="93"/>
+      <c r="C2" s="93"/>
+      <c r="D2" s="93"/>
+      <c r="E2" s="93"/>
+      <c r="F2" s="93"/>
+      <c r="G2" s="93"/>
+      <c r="H2" s="93"/>
     </row>
     <row r="4" spans="1:8" ht="39.75" customHeight="1">
-      <c r="A4" s="91" t="s">
+      <c r="A4" s="92" t="s">
         <v>425</v>
       </c>
-      <c r="B4" s="92"/>
-      <c r="C4" s="92"/>
-      <c r="D4" s="92"/>
-      <c r="E4" s="92"/>
-      <c r="F4" s="92"/>
-      <c r="G4" s="92"/>
-      <c r="H4" s="92"/>
+      <c r="B4" s="93"/>
+      <c r="C4" s="93"/>
+      <c r="D4" s="93"/>
+      <c r="E4" s="93"/>
+      <c r="F4" s="93"/>
+      <c r="G4" s="93"/>
+      <c r="H4" s="93"/>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
       <c r="A6" s="48" t="s">
@@ -5565,7 +5569,7 @@
       <c r="F5" s="58" t="s">
         <v>503</v>
       </c>
-      <c r="G5" s="94" t="s">
+      <c r="G5" s="95" t="s">
         <v>504</v>
       </c>
       <c r="H5" s="61">
@@ -5604,7 +5608,7 @@
       <c r="F6" s="58" t="s">
         <v>505</v>
       </c>
-      <c r="G6" s="95"/>
+      <c r="G6" s="96"/>
       <c r="J6" s="60">
         <f t="shared" ca="1" si="2"/>
         <v>14</v>
@@ -5633,7 +5637,7 @@
       <c r="F7" s="58" t="s">
         <v>506</v>
       </c>
-      <c r="G7" s="94" t="s">
+      <c r="G7" s="95" t="s">
         <v>507</v>
       </c>
       <c r="H7" s="61">
@@ -5668,7 +5672,7 @@
       <c r="F8" s="58" t="s">
         <v>508</v>
       </c>
-      <c r="G8" s="95"/>
+      <c r="G8" s="96"/>
       <c r="J8" s="60">
         <f t="shared" ca="1" si="2"/>
         <v>4.8</v>
@@ -5697,7 +5701,7 @@
       <c r="F9" s="58" t="s">
         <v>509</v>
       </c>
-      <c r="G9" s="95"/>
+      <c r="G9" s="96"/>
       <c r="J9" s="60">
         <f t="shared" ca="1" si="2"/>
         <v>3.9</v>
@@ -5726,7 +5730,7 @@
       <c r="F10" s="58" t="s">
         <v>510</v>
       </c>
-      <c r="G10" s="95"/>
+      <c r="G10" s="96"/>
       <c r="J10" s="60">
         <f t="shared" ca="1" si="2"/>
         <v>13.6</v>
@@ -5936,7 +5940,7 @@
       <c r="F17" s="58" t="s">
         <v>517</v>
       </c>
-      <c r="G17" s="94" t="s">
+      <c r="G17" s="95" t="s">
         <v>26</v>
       </c>
       <c r="H17" s="61">
@@ -5971,7 +5975,7 @@
       <c r="F18" s="58" t="s">
         <v>518</v>
       </c>
-      <c r="G18" s="95"/>
+      <c r="G18" s="96"/>
       <c r="J18" s="60">
         <f t="shared" ca="1" si="2"/>
         <v>3.9</v>
@@ -6495,8 +6499,8 @@
       <c r="A13" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="B13" s="96">
-        <v>46262</v>
+      <c r="B13" s="91">
+        <v>46258</v>
       </c>
       <c r="C13" s="16">
         <f t="shared" si="0"/>

</xml_diff>